<commit_message>
fix(docs): correct pipeline run command to include --dataset-config
default.yaml lacks the dataset key on its own; the runnable command pairs it
with a dataset config (cityflowv2 / wildtrack). Verified via --dry-run.
Update README.md and the Excel run instructions.
</commit_message>
<xml_diff>
--- a/Project Code.xlsx
+++ b/Project Code.xlsx
@@ -675,7 +675,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Requires Python 3.10-3.13. Create a virtual environment and run 'pip install -r requirements.txt'. Download model weights with 'python scripts/download_weights.py --set all' and verify them with 'python scripts/verify_assets.py'. Run the pipeline with 'python scripts/run_pipeline.py --config configs/default.yaml' (add '--smoke-test' for a quick run on the first frames). The datasets (CityFlowV2, WILDTRACK, VeRi-776) are large and external; download them separately as described in README.md. To launch the live app, start the backend with 'python -m uvicorn backend_api:app --port 8000' and the frontend with 'cd frontend &amp;&amp; npm install &amp;&amp; npm run dev' (opens on http://127.0.0.1:3001). Run the tests with 'pytest tests/'. Full instructions are in README.md, SETUP.md, and LAUNCH.md.</t>
+          <t>Requires Python 3.10-3.13. Create a virtual environment and run 'pip install -r requirements.txt'. Download model weights with 'python scripts/download_weights.py --set all' and verify them with 'python scripts/verify_assets.py'. Run the pipeline with 'python scripts/run_pipeline.py --config configs/default.yaml --dataset-config configs/datasets/cityflowv2.yaml' (add '--smoke-test' for a quick run on the first frames, or '--dataset-config configs/datasets/wildtrack.yaml' for the person pipeline). The datasets (CityFlowV2, WILDTRACK, VeRi-776) are large and external; download them separately as described in README.md. To launch the live app, start the backend with 'python -m uvicorn backend_api:app --port 8000' and the frontend with 'cd frontend &amp;&amp; npm install &amp;&amp; npm run dev' (opens on http://127.0.0.1:3001). Run the tests with 'pytest tests/'. Full instructions are in README.md, SETUP.md, and LAUNCH.md.</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,6 @@
           <t>Original</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11" ht="64" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
@@ -766,7 +765,6 @@
           <t>Original</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12" ht="64" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
@@ -894,7 +892,6 @@
           <t>Original</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -956,7 +953,6 @@
           <t>Original</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -974,7 +970,6 @@
           <t>Original</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1058,7 +1053,6 @@
           <t>Original</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1076,7 +1070,6 @@
           <t>Original</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1094,7 +1087,6 @@
           <t>Original</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1134,7 +1126,6 @@
           <t>Original</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1234,7 +1225,6 @@
           <t>Shared data models, config loading, IO utilities, constants.</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1257,7 +1247,6 @@
           <t>Frame extraction and preprocessing.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1415,7 +1404,6 @@
           <t>Annotated video, BEV, and timeline outputs.</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1492,7 +1480,6 @@
           <t>ReID model loaders and model cache.</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1515,7 +1502,6 @@
           <t>Streamlit dashboard, NL query, 3D simulation.</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1619,7 +1605,6 @@
           <t>OmegaConf pipeline/dataset/model configs and registry.</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1642,7 +1627,6 @@
           <t>CLI entry points, asset download/verify, evaluation helpers.</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1665,7 +1649,6 @@
           <t>Pytest suite across stages, backend, and scripts.</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1715,7 +1698,6 @@
           <t>Architecture, dataset, and model-card reference docs.</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1765,7 +1747,6 @@
           <t>Top-level README, SETUP, and LAUNCH guides.</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1788,7 +1769,6 @@
           <t>MIT license.</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1838,7 +1818,6 @@
           <t>Build config and project metadata.</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1861,7 +1840,6 @@
           <t>Setuptools shim.</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1884,7 +1862,6 @@
           <t>Convenience make targets.</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1907,7 +1884,6 @@
           <t>App launchers (Python/shell/batch).</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1930,7 +1906,6 @@
           <t>Backend ASGI entry point.</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1953,7 +1928,6 @@
           <t>Utility to free the backend port.</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1976,7 +1950,6 @@
           <t>GitHub Actions CI workflow.</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1999,7 +1972,6 @@
           <t>Git ignore rules.</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
docs(submission): refine Project Code.xlsx source categorization
Mark all team-authored code "Original" with Comments disclosing adapted/ported/
glued parts (transreid_model, clip_senet_model, stage4/fic, training/losses,
training/model adapted from upstream; stage1/3/5 + serving are library glue).
Keep shadcn/ui and CityFlowV2 ground-truth as "Copied"; LICENSE and the sheet
itself as "Original from Template". Verified 100% file coverage (410 tracked
files across 40 rows).
</commit_message>
<xml_diff>
--- a/Project Code.xlsx
+++ b/Project Code.xlsx
@@ -784,7 +784,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Wraps the external ultralytics and boxmot libraries (pip dependencies).</t>
+          <t>Wrappers/glue around Ultralytics YOLO and BoxMOT (BoT-SORT).</t>
         </is>
       </c>
     </row>
@@ -806,7 +806,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Model implementations cite their source papers in the file headers.</t>
+          <t>Mostly bespoke; transreid_model.py and clip_senet_model.py adapt/port upstream ReID architectures (see Files sheet).</t>
         </is>
       </c>
     </row>
@@ -828,7 +828,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Wraps the external faiss library.</t>
+          <t>Wrapper/glue around FAISS and SQLite.</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Algorithm implementations cite their source papers.</t>
+          <t>Bespoke association algorithms; fic.py adapted from the AIC21 1st-place ficfac.py (see Files sheet).</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Wraps the external trackeval and motmetrics libraries.</t>
+          <t>Wrapper/glue around TrackEval and py-motmetrics.</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Loss implementations cite their source papers.</t>
+          <t>Bespoke trainer; losses.py and model.py adapt canonical BoT / IBN-Net reference code (see Files sheet).</t>
         </is>
       </c>
     </row>
@@ -953,6 +953,11 @@
           <t>Original</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Loaders/glue around torch / timm / open_clip checkpoints.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1033,7 +1038,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Generated from the shadcn/ui component library.</t>
+          <t>Generated by the shadcn/ui CLI - not written by us.</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="91.1796875" customWidth="1" min="1" max="1"/>
@@ -1247,6 +1252,11 @@
           <t>Frame extraction and preprocessing.</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Uses OpenCV.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1271,7 +1281,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Wraps ultralytics and boxmot (pip dependencies).</t>
+          <t>Glue/wrappers around Ultralytics YOLO and BoxMOT (BoT-SORT); the BoxMOT numpy-array KF patch is ours.</t>
         </is>
       </c>
     </row>
@@ -1298,19 +1308,19 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>TransReID/CLIP-SENet model code cites source papers in headers.</t>
+          <t>Bespoke except the two model files below; pca_whitening wraps scikit-learn PCA, hsv_extractor uses OpenCV.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>src/stage3_indexing/**/*</t>
+          <t>src/stage2_features/transreid_model.py</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Stage 3 - Indexing</t>
+          <t>Stage 2 - Features</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1320,24 +1330,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>FAISS index and SQLite metadata.</t>
+          <t>TransReID model for inference.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Wraps the faiss library.</t>
+          <t>ADAPTED: SIE/JPM/BNNeck follow the official TransReID architecture (He et al., ICCV 2021) on a timm/CLIP backbone.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>src/stage4_association/**/*</t>
+          <t>src/stage2_features/clip_senet_model.py</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Stage 4 - Association</t>
+          <t>Stage 2 - Features</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1347,24 +1357,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Cross-camera association graph and solver.</t>
+          <t>CLIP-SENet vehicle ReID model.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AQE/FIC/k-reciprocal-rerank implementations cite source papers.</t>
+          <t>PORT of the CLIP-SENet architecture (AFEM) from the paper; backbones (ResNet101-IBN via XingangPan/IBN-Net, TinyCLIP) loaded via torch.hub / open_clip.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>src/stage5_evaluation/**/*</t>
+          <t>src/stage3_indexing/**/*</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Stage 5 - Evaluation</t>
+          <t>Stage 3 - Indexing</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1374,24 +1384,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Metrics and MOTChallenge format conversion.</t>
+          <t>FAISS index and SQLite metadata.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Wraps trackeval and motmetrics.</t>
+          <t>Glue/wrapper around FAISS and SQLite.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>src/stage6_visualization/**/*</t>
+          <t>src/stage4_association/**/*</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Stage 6 - Visualization</t>
+          <t>Stage 4 - Association</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1401,19 +1411,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Annotated video, BEV, and timeline outputs.</t>
+          <t>Cross-camera association graph and solver.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Bespoke; AQE/k-reciprocal-rerank/camera-bias cite their source papers in headers; graph_solver uses networkx + scikit-learn + scipy.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>src/stage_wildtrack_mvdetr/**/*</t>
+          <t>src/stage4_association/fic.py</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>WILDTRACK MVDeTr</t>
+          <t>Stage 4 - Association</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1423,24 +1438,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Ground-plane person detection and tracking path.</t>
+          <t>Per-camera feature-improvement whitening.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Integrates the MVDeTr method.</t>
+          <t>ADAPTED from the AIC21 1st-place solution ficfac.py (Liu et al., CVPRW 2021).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>src/training/**/*</t>
+          <t>src/stage5_evaluation/**/*</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ReID Training</t>
+          <t>Stage 5 - Evaluation</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1450,24 +1465,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Training loops, losses, dataset builders.</t>
+          <t>Metrics and MOTChallenge format conversion.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Loss implementations cite source papers.</t>
+          <t>Glue/wrapper around TrackEval and py-motmetrics.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>src/serving/**/*</t>
+          <t>src/stage6_visualization/**/*</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Model Serving</t>
+          <t>Stage 6 - Visualization</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1477,19 +1492,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ReID model loaders and model cache.</t>
+          <t>Annotated video, BEV, and timeline outputs.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Uses OpenCV for drawing.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>src/apps/**/*</t>
+          <t>src/stage_wildtrack_mvdetr/**/*</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Auxiliary Apps</t>
+          <t>WILDTRACK MVDeTr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1499,19 +1519,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Streamlit dashboard, NL query, 3D simulation.</t>
+          <t>Ground-plane person detection and tracking path.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Bespoke Kalman tracker + integration glue; consumes external MVDeTr detector outputs.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>backend/**/*</t>
+          <t>src/training/**/*</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Backend API</t>
+          <t>ReID Training</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1521,51 +1546,51 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>FastAPI service, routers, services, model registry.</t>
+          <t>Training loops, losses, dataset builders.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Built on FastAPI (pip dependency).</t>
+          <t>Bespoke trainer/datasets except the two files below.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>frontend/src/components/ui/**/*</t>
+          <t>src/training/losses.py</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Frontend UI Primitives</t>
+          <t>ReID Training</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Copied</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Reusable UI primitives (button, dialog, tabs, etc.).</t>
+          <t>ReID loss functions.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Generated from shadcn/ui (https://ui.shadcn.com/), built on Radix UI.</t>
+          <t>ADAPTED from the canonical 'Bag of Tricks' reference implementations (Luo et al., reid-strong-baseline; Center loss from Wen et al., ECCV 2016).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>frontend/**/*</t>
+          <t>src/training/model.py</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Frontend Dashboard</t>
+          <t>ReID Training</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1575,24 +1600,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Next.js ATHAR dashboard app, hooks, store, API client.</t>
+          <t>BoT ReID backbone.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Excludes src/components/ui/** (see the Copied row above). Uses Next.js/React/Tailwind (npm dependencies).</t>
+          <t>ADAPTED: IBN-a layer follows XingangPan/IBN-Net; BNNeck baseline follows BoT (Luo et al., CVPRW 2019); loads IBN-Net pretrained weights by URL.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>configs/**/*</t>
+          <t>src/serving/**/*</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Configuration</t>
+          <t>Model Serving</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1602,19 +1627,24 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>OmegaConf pipeline/dataset/model configs and registry.</t>
+          <t>ReID model loaders and model cache.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Loaders/glue around torch / timm / open_clip checkpoints.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>scripts/**/*</t>
+          <t>src/apps/**/*</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Auxiliary Apps</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1624,19 +1654,19 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CLI entry points, asset download/verify, evaluation helpers.</t>
+          <t>Streamlit dashboard, NL query, 3D simulation.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>tests/**/*</t>
+          <t>backend/**/*</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Tests</t>
+          <t>Backend API</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1646,46 +1676,51 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Pytest suite across stages, backend, and scripts.</t>
+          <t>FastAPI service, routers, services, model registry.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Built on the FastAPI framework.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>notebooks/**/*</t>
+          <t>frontend/src/components/ui/**/*</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Kaggle Notebooks</t>
+          <t>Frontend UI Primitives</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Original from Template</t>
+          <t>Copied</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>GPU training, pipeline, and verification runners for Kaggle.</t>
+          <t>Reusable UI primitives (button, dialog, tabs, etc.).</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Generated from templates by the project's notebook-builder tooling; wrap the pipeline code under src/.</t>
+          <t>Generated by the shadcn/ui CLI (https://ui.shadcn.com/), built on Radix UI - not written by us.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>docs/**/*</t>
+          <t>frontend/**/*</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Frontend Dashboard</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1695,46 +1730,51 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Architecture, dataset, and model-card reference docs.</t>
+          <t>Next.js ATHAR dashboard app, hooks, store, API client.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Excludes src/components/ui/** (shadcn, see the Copied row). Root config (next.config, tsconfig, tailwind.config, components.json, package.json) was scaffolded by create-next-app + shadcn init and customized by us; next-env.d.ts and package-lock.json are auto-generated.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>data/raw/cityflowv2/**/*</t>
+          <t>configs/**/*</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Datasets (ground truth)</t>
+          <t>Configuration</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Copied</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>CityFlowV2 ground-truth and seqinfo files for evaluation.</t>
+          <t>OmegaConf pipeline/dataset/model configs and registry.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>From the CityFlowV2 / AI City Challenge 2022 dataset (external; full dataset not included).</t>
+          <t>Hand-tuned.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>*.md</t>
+          <t>scripts/**/*</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Scripts and Tooling</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1744,19 +1784,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Top-level README, SETUP, and LAUNCH guides.</t>
+          <t>CLI entry points, asset download/verify, evaluation helpers.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>scripts/eval/ modules wrap the ReID models for VeRi-776 evaluation.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>LICENSE</t>
+          <t>tests/**/*</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Tests</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1766,19 +1811,19 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MIT license.</t>
+          <t>Pytest suite across stages, backend, and scripts.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>*requirements.txt</t>
+          <t>notebooks/**/*</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Kaggle Notebooks</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1788,24 +1833,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Python dependency manifests.</t>
+          <t>GPU training, pipeline, and verification runners for Kaggle.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>List external pip dependencies (not vendored).</t>
+          <t>Generated from templates by the project's own notebook-builder tooling; they wrap the pipeline code under src/.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>pyproject.toml</t>
+          <t>docs/**/*</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1815,19 +1860,19 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Build config and project metadata.</t>
+          <t>Architecture, dataset, and model-card reference docs.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>setup.py</t>
+          <t>*.md</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1837,36 +1882,41 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Setuptools shim.</t>
+          <t>Top-level README, SETUP, and LAUNCH guides.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Makefile</t>
+          <t>LICENSE</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Original from Template</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Convenience make targets.</t>
+          <t>MIT license.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Standard MIT License text.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>start.*</t>
+          <t>*requirements.txt</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1881,14 +1931,19 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>App launchers (Python/shell/batch).</t>
+          <t>Python dependency manifests.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>List external pip dependencies (not vendored).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>backend_api.py</t>
+          <t>pyproject.toml</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1903,14 +1958,14 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Backend ASGI entry point.</t>
+          <t>Build config and project metadata.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>kill_backend.py</t>
+          <t>setup.py</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1925,14 +1980,14 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Utility to free the backend port.</t>
+          <t>Setuptools shim.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>.github/**/*</t>
+          <t>Makefile</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1947,29 +2002,221 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>GitHub Actions CI workflow.</t>
+          <t>Convenience make targets.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>start.*</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>App launchers (Python/shell/batch).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>backend_api.py</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Backend ASGI entry point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>kill_backend.py</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Utility to free the backend port.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>.github/**/*</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>GitHub Actions CI workflow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>.gitignore</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>Scripts and Tooling</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Original</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
         <is>
           <t>Git ignore rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>data/raw/cityflowv2/**/*</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Datasets (ground truth)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Copied</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>CityFlowV2 ground-truth and seqinfo files for evaluation.</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>From the external CityFlowV2 / AI City Challenge 2022 dataset (full dataset not included).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>src/__init__.py</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Top-level src package marker.</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>models/**/*</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Model-weights README and placement/checksum instructions.</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>The checkpoints themselves are large and not included (gitignored); see README for download/generation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Project Code.xlsx</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Original from Template</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>This submission spreadsheet.</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Course-provided template, filled in by us.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(submission): provenance re-audit of Project Code.xlsx sources
Deep audit of all bespoke files. Reclassify files containing canonical/
reference code: losses.py + use-toast.ts -> Copied; transreid_model,
clip_senet_model, fic, model, evaluate_reid, preprocessor (CLAHE),
foreground_mask*, reid_service (k-reciprocal), lib/utils.ts, scripts/eval
-> Mixed (bespoke + external, detailed in comments). reranking.py and
aflink.py verified bespoke (not canonical ports). Standard textbook/library
idioms (Kalman, calibration, IoU, CLIP constants, PK sampler) kept Original
with disclosure comments. 100% file coverage (48 rows / 410 files).
</commit_message>
<xml_diff>
--- a/Project Code.xlsx
+++ b/Project Code.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="29.54296875" customWidth="1" min="1" max="1"/>
@@ -765,6 +765,11 @@
           <t>Original</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Bespoke; preprocessor CLAHE follows the OpenCV tutorial recipe; format_converter follows MOT/WILDTRACK schemas.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="64" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
@@ -784,7 +789,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Wrappers/glue around Ultralytics YOLO and BoxMOT (BoT-SORT).</t>
+          <t>Wrappers/glue around Ultralytics YOLO and BoxMOT (BoT-SORT); IoU/interpolation are textbook helpers.</t>
         </is>
       </c>
     </row>
@@ -806,7 +811,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Mostly bespoke; transreid_model.py and clip_senet_model.py adapt/port upstream ReID architectures (see Files sheet).</t>
+          <t>Mostly bespoke; transreid_model + clip_senet_model adapt upstream architectures; SAM2 maskers follow the SAM2 model-card usage (see Files sheet).</t>
         </is>
       </c>
     </row>
@@ -850,7 +855,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Bespoke association algorithms; fic.py adapted from the AIC21 1st-place ficfac.py (see Files sheet).</t>
+          <t>Bespoke reimplementations (reranking/aflink verified not ports); fic.py adapted from AIC21 ficfac.py.</t>
         </is>
       </c>
     </row>
@@ -911,7 +916,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Integrates the MVDeTr multi-view detection method.</t>
+          <t>Bespoke integration glue; textbook constant-velocity Kalman tracker; consumes external MVDeTr outputs.</t>
         </is>
       </c>
     </row>
@@ -933,7 +938,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Bespoke trainer; losses.py and model.py adapt canonical BoT / IBN-Net reference code (see Files sheet).</t>
+          <t>Bespoke trainer; losses.py copied + model.py/evaluate_reid.py adapt canonical BoT / Market-1501 reference code (see Files sheet).</t>
         </is>
       </c>
     </row>
@@ -955,7 +960,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Loaders/glue around torch / timm / open_clip checkpoints.</t>
+          <t>Loaders/glue around torch / timm / open_clip; standard CLIP/ImageNet normalization constants.</t>
         </is>
       </c>
     </row>
@@ -994,7 +999,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Built on the FastAPI framework (pip dependency).</t>
+          <t>Bespoke FastAPI app; reid_service.py contains the canonical k-reciprocal re-ranking algorithm (see Files sheet).</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1021,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Built on Next.js, React, and Tailwind (npm dependencies).</t>
+          <t>Bespoke Next.js app; use-toast.ts copied from shadcn and lib/utils.ts has common helper snippets (see Files sheet).</t>
         </is>
       </c>
     </row>
@@ -1075,6 +1080,11 @@
           <t>Original</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Bespoke CLI/tooling; scripts/eval/ contains canonical k-reciprocal + Market-1501 eval reference code (see Files sheet).</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1154,6 +1164,15 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A8:D8"/>
@@ -1172,7 +1191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="91.1796875" customWidth="1" min="1" max="1"/>
@@ -1212,7 +1231,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>src/core/**/*</t>
+          <t>src/__init__.py</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1227,19 +1246,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Shared data models, config loading, IO utilities, constants.</t>
-        </is>
-      </c>
+          <t>Top-level src package marker.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>src/stage0_ingestion/**/*</t>
+          <t>src/core/**/*</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Stage 0 - Ingestion</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1249,24 +1269,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Frame extraction and preprocessing.</t>
+          <t>Shared data models, config loading, IO utilities.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Uses OpenCV.</t>
+          <t>Bespoke; io_utils numpy-JSON encoder, video_utils FourCC decode, and wildtrack_calibration (cv2 projectPoints/Rodrigues + WILDTRACK grid) use standard OpenCV/numpy idioms.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>src/stage1_tracking/**/*</t>
+          <t>src/stage0_ingestion/**/*</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Stage 1 - Tracking</t>
+          <t>Stage 0 - Ingestion</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1276,51 +1296,51 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>YOLO detection and BoxMOT single-camera tracking.</t>
+          <t>Frame extraction and preprocessing.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Glue/wrappers around Ultralytics YOLO and BoxMOT (BoT-SORT); the BoxMOT numpy-array KF patch is ours.</t>
+          <t>Bespoke; format_converter follows the MOTChallenge/WILDTRACK annotation schemas.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>src/stage2_features/**/*</t>
+          <t>src/stage0_ingestion/preprocessor.py</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Stage 2 - Features</t>
+          <t>Stage 0 - Ingestion</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ReID embeddings, HSV histograms, PCA whitening.</t>
+          <t>Frame preprocessing (CLAHE, denoise).</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Bespoke except the two model files below; pca_whitening wraps scikit-learn PCA, hsv_extractor uses OpenCV.</t>
+          <t>MIXED: the LAB-channel CLAHE block follows the canonical OpenCV tutorial recipe; surrounding pipeline is bespoke.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>src/stage2_features/transreid_model.py</t>
+          <t>src/stage1_tracking/**/*</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Stage 2 - Features</t>
+          <t>Stage 1 - Tracking</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1330,19 +1350,19 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>TransReID model for inference.</t>
+          <t>YOLO detection + BoxMOT tracking.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ADAPTED: SIE/JPM/BNNeck follow the official TransReID architecture (He et al., ICCV 2021) on a timm/CLIP backbone.</t>
+          <t>Glue/wrappers around Ultralytics YOLO and BoxMOT (BoT-SORT); IoU + linear interpolation are textbook helpers; rest bespoke.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>src/stage2_features/clip_senet_model.py</t>
+          <t>src/stage2_features/**/*</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1357,132 +1377,132 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CLIP-SENet vehicle ReID model.</t>
+          <t>ReID embeddings, HSV, PCA.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PORT of the CLIP-SENet architecture (AFEM) from the paper; backbones (ResNet101-IBN via XingangPan/IBN-Net, TinyCLIP) loaded via torch.hub / open_clip.</t>
+          <t>Bespoke; pca_whitening wraps sklearn PCA, hsv_extractor uses cv2.calcHist, reid_model state-dict remaps are keyed to fast-reid/IBN-Net layouts.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>src/stage3_indexing/**/*</t>
+          <t>src/stage2_features/transreid_model.py</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Stage 3 - Indexing</t>
+          <t>Stage 2 - Features</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>FAISS index and SQLite metadata.</t>
+          <t>TransReID model for inference.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Glue/wrapper around FAISS and SQLite.</t>
+          <t>MIXED: SIE/JPM/BNNeck follow the official TransReID architecture (He et al., ICCV 2021); timm/CLIP integration + weight remapping bespoke.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>src/stage4_association/**/*</t>
+          <t>src/stage2_features/clip_senet_model.py</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Stage 4 - Association</t>
+          <t>Stage 2 - Features</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Cross-camera association graph and solver.</t>
+          <t>CLIP-SENet vehicle ReID model.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Bespoke; AQE/k-reciprocal-rerank/camera-bias cite their source papers in headers; graph_solver uses networkx + scikit-learn + scipy.</t>
+          <t>MIXED: AFEM/architecture ported from the CLIP-SENet paper; backbones via torch.hub/open_clip; assembly bespoke.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>src/stage4_association/fic.py</t>
+          <t>src/stage2_features/foreground_masker.py</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Stage 4 - Association</t>
+          <t>Stage 2 - Features</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Per-camera feature-improvement whitening.</t>
+          <t>SAM2 foreground masking.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ADAPTED from the AIC21 1st-place solution ficfac.py (Liu et al., CVPRW 2021).</t>
+          <t>MIXED: SAM2 point-prompt inference follows the official SAM2 model-card usage; registry/loader bespoke (default-off experimental).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>src/stage5_evaluation/**/*</t>
+          <t>src/stage2_features/foreground_masking.py</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Stage 5 - Evaluation</t>
+          <t>Stage 2 - Features</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Metrics and MOTChallenge format conversion.</t>
+          <t>SAM2 automatic-mask masking.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Glue/wrapper around TrackEval and py-motmetrics.</t>
+          <t>MIXED: SAM2 automatic-mask-generator usage from the SAM2 README; plumbing bespoke (default-off experimental).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>src/stage6_visualization/**/*</t>
+          <t>src/stage3_indexing/**/*</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Stage 6 - Visualization</t>
+          <t>Stage 3 - Indexing</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1492,24 +1512,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Annotated video, BEV, and timeline outputs.</t>
+          <t>FAISS index and SQLite metadata.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Uses OpenCV for drawing.</t>
+          <t>Glue/wrapper around FAISS + SQLite (idiomatic API usage).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>src/stage_wildtrack_mvdetr/**/*</t>
+          <t>src/stage4_association/**/*</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>WILDTRACK MVDeTr</t>
+          <t>Stage 4 - Association</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1519,51 +1539,51 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Ground-plane person detection and tracking path.</t>
+          <t>Cross-camera association graph and solver.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Bespoke Kalman tracker + integration glue; consumes external MVDeTr detector outputs.</t>
+          <t>Bespoke reimplementations; AQE/k-reciprocal/AFLink/camera-bias/zone cite their techniques in headers (verified not line-level ports).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>src/training/**/*</t>
+          <t>src/stage4_association/fic.py</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ReID Training</t>
+          <t>Stage 4 - Association</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Training loops, losses, dataset builders.</t>
+          <t>Per-camera FIC whitening.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Bespoke trainer/datasets except the two files below.</t>
+          <t>MIXED: per-camera whitening adapted from the AIC21 1st-place ficfac.py (Liu et al., CVPRW 2021); wrappers bespoke.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>src/training/losses.py</t>
+          <t>src/stage5_evaluation/**/*</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ReID Training</t>
+          <t>Stage 5 - Evaluation</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1573,24 +1593,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>ReID loss functions.</t>
+          <t>Metrics and format conversion.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ADAPTED from the canonical 'Bag of Tricks' reference implementations (Luo et al., reid-strong-baseline; Center loss from Wen et al., ECCV 2016).</t>
+          <t>Glue/wrapper around TrackEval + py-motmetrics.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>src/training/model.py</t>
+          <t>src/stage6_visualization/**/*</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ReID Training</t>
+          <t>Stage 6 - Visualization</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1600,24 +1620,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>BoT ReID backbone.</t>
+          <t>Annotated video, BEV, timeline.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ADAPTED: IBN-a layer follows XingangPan/IBN-Net; BNNeck baseline follows BoT (Luo et al., CVPRW 2019); loads IBN-Net pretrained weights by URL.</t>
+          <t>Bespoke; standard matplotlib/Plotly palettes and cv2 drawing idioms.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>src/serving/**/*</t>
+          <t>src/stage_wildtrack_mvdetr/**/*</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Model Serving</t>
+          <t>WILDTRACK MVDeTr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1627,24 +1647,24 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ReID model loaders and model cache.</t>
+          <t>Ground-plane person detection + tracking.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Loaders/glue around torch / timm / open_clip checkpoints.</t>
+          <t>Bespoke glue; constant-velocity Kalman is the textbook DWNA model; WILDTRACK grid constants are dataset facts; consumes external MVDeTr outputs.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>src/apps/**/*</t>
+          <t>src/training/**/*</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Auxiliary Apps</t>
+          <t>ReID Training</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1654,100 +1674,105 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Streamlit dashboard, NL query, 3D simulation.</t>
+          <t>Training loops, datasets, seeding.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Bespoke trainer; datasets/seed/train_reid follow the standard BoT recipe + PyTorch reproducibility idioms (independently written). See per-file rows.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>backend/**/*</t>
+          <t>src/training/losses.py</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Backend API</t>
+          <t>ReID Training</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Copied</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>FastAPI service, routers, services, model registry.</t>
+          <t>ReID loss functions.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Built on the FastAPI framework.</t>
+          <t>COPIED: Triplet/Center/CE-label-smoothing/Circle losses follow the canonical BoT reference implementations (Luo et al. reid-strong-baseline; Center loss Wen et al.).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>frontend/src/components/ui/**/*</t>
+          <t>src/training/model.py</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Frontend UI Primitives</t>
+          <t>ReID Training</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Copied</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Reusable UI primitives (button, dialog, tabs, etc.).</t>
+          <t>BoT ReID backbone.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Generated by the shadcn/ui CLI (https://ui.shadcn.com/), built on Radix UI - not written by us.</t>
+          <t>MIXED: IBN-a from XingangPan/IBN-Net + BNNeck from BoT (canonical); build/loading bespoke; loads IBN-Net weights by URL.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>frontend/**/*</t>
+          <t>src/training/evaluate_reid.py</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Frontend Dashboard</t>
+          <t>ReID Training</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Next.js ATHAR dashboard app, hooks, store, API client.</t>
+          <t>ReID evaluation (CMC/mAP) + re-ranking.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Excludes src/components/ui/** (shadcn, see the Copied row). Root config (next.config, tsconfig, tailwind.config, components.json, package.json) was scaffolded by create-next-app + shadcn init and customized by us; next-env.d.ts and package-lock.json are auto-generated.</t>
+          <t>MIXED: eval_market1501 (CMC/mAP) and compute_reranking (k-reciprocal, Zhong et al. 2017) follow canonical Market-1501/reid reference code; orchestration bespoke.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>configs/**/*</t>
+          <t>src/serving/**/*</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Configuration</t>
+          <t>Model Serving</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1757,24 +1782,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>OmegaConf pipeline/dataset/model configs and registry.</t>
+          <t>ReID model loaders and cache.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Hand-tuned.</t>
+          <t>Loaders/glue around torch/timm/open_clip; CLIP/ImageNet normalization are the standard published constants.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>scripts/**/*</t>
+          <t>src/apps/**/*</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Auxiliary Apps</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1784,24 +1809,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>CLI entry points, asset download/verify, evaluation helpers.</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>scripts/eval/ modules wrap the ReID models for VeRi-776 evaluation.</t>
-        </is>
-      </c>
+          <t>Streamlit dashboard, NL query, 3D sim.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>tests/**/*</t>
+          <t>backend/**/*</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tests</t>
+          <t>Backend API</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1811,117 +1832,132 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Pytest suite across stages, backend, and scripts.</t>
+          <t>FastAPI service, routers, services, registry.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Bespoke FastAPI application (framework idioms are normal usage).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>notebooks/**/*</t>
+          <t>backend/services/reid_service.py</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Kaggle Notebooks</t>
+          <t>Backend API</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>GPU training, pipeline, and verification runners for Kaggle.</t>
+          <t>ReID inference service.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Generated from templates by the project's own notebook-builder tooling; they wrap the pipeline code under src/.</t>
+          <t>MIXED: the dense _compute_reranking is the canonical k-reciprocal algorithm (Zhong et al. 2017); image handling/AQE/fusion/scoring bespoke.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>docs/**/*</t>
+          <t>frontend/src/components/ui/**/*</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Frontend UI Primitives</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Copied</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Architecture, dataset, and model-card reference docs.</t>
+          <t>Reusable UI primitives.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Generated by the shadcn/ui CLI (https://ui.shadcn.com/), built on Radix UI - not written by us.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>*.md</t>
+          <t>frontend/src/hooks/use-toast.ts</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Frontend Dashboard</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Copied</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Top-level README, SETUP, and LAUNCH guides.</t>
+          <t>Toast notification hook.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>COPIED: the shadcn/ui use-toast hook (adapted from react-hot-toast).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>LICENSE</t>
+          <t>frontend/src/lib/utils.ts</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Frontend Dashboard</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Original from Template</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>MIT license.</t>
+          <t>Frontend utility helpers.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Standard MIT License text.</t>
+          <t>MIXED: cn() (shadcn), debounce/throttle/formatBytes/getCameraColor are common tutorial/Stack-Overflow snippets; other helpers bespoke.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>*requirements.txt</t>
+          <t>frontend/**/*</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Frontend Dashboard</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1931,24 +1967,24 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Python dependency manifests.</t>
+          <t>Next.js ATHAR dashboard app, hooks, store, API client.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>List external pip dependencies (not vendored).</t>
+          <t>Excludes components/ui/** and the two files above. Root config (next.config, tsconfig, tailwind, components.json, package.json) scaffolded by create-next-app + shadcn init and customized by us; next-env.d.ts/package-lock.json auto-generated.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>pyproject.toml</t>
+          <t>configs/**/*</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Configuration</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1958,14 +1994,19 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Build config and project metadata.</t>
+          <t>OmegaConf pipeline/dataset/model configs.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Hand-tuned.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>setup.py</t>
+          <t>scripts/**/*</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1980,14 +2021,19 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Setuptools shim.</t>
+          <t>CLI entry points, asset download/verify, helpers.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Bespoke; see scripts/eval row.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Makefile</t>
+          <t>scripts/eval/**/*</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1997,24 +2043,29 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Convenience make targets.</t>
+          <t>VeRi-776 ReID evaluation modules.</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>MIXED: compute_reranking_torch (k-reciprocal, Zhong et al. 2017) and eval_market1501 (CMC/mAP) are canonical ReID reference code; model defs + CLI/JSON plumbing bespoke.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>start.*</t>
+          <t>tests/**/*</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Tests</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2024,41 +2075,47 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>App launchers (Python/shell/batch).</t>
-        </is>
-      </c>
+          <t>Pytest suite across stages, backend, scripts.</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>backend_api.py</t>
+          <t>notebooks/**/*</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Kaggle Notebooks</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Original from Template</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Backend ASGI entry point.</t>
+          <t>GPU training/pipeline/verification runners.</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Generated from templates by the project's notebook-builder tooling; wrap src/ pipeline code.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>kill_backend.py</t>
+          <t>docs/**/*</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2068,19 +2125,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Utility to free the backend port.</t>
-        </is>
-      </c>
+          <t>Architecture, dataset, model-card docs.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>.github/**/*</t>
+          <t>*.md</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2090,91 +2148,101 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>GitHub Actions CI workflow.</t>
-        </is>
-      </c>
+          <t>Top-level README, SETUP, LAUNCH guides.</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>.gitignore</t>
+          <t>LICENSE</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Original from Template</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Git ignore rules.</t>
+          <t>MIT license.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Standard MIT License text.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>data/raw/cityflowv2/**/*</t>
+          <t>models/**/*</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Datasets (ground truth)</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Copied</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>CityFlowV2 ground-truth and seqinfo files for evaluation.</t>
+          <t>Model-weights README / placement instructions.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>From the external CityFlowV2 / AI City Challenge 2022 dataset (full dataset not included).</t>
+          <t>Checkpoints themselves are not included (gitignored); see README.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>src/__init__.py</t>
+          <t>Project Code.xlsx</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Original from Template</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Top-level src package marker.</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr"/>
+          <t>This submission spreadsheet.</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Course-provided template, filled in by us.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>models/**/*</t>
+          <t>*requirements.txt</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Scripts and Tooling</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2184,39 +2252,223 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Model-weights README and placement/checksum instructions.</t>
+          <t>Python dependency manifests.</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>The checkpoints themselves are large and not included (gitignored); see README for download/generation.</t>
+          <t>List external pip dependencies (not vendored).</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Project Code.xlsx</t>
+          <t>pyproject.toml</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Scripts and Tooling</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Original from Template</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>This submission spreadsheet.</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Course-provided template, filled in by us.</t>
+          <t>Build config and project metadata.</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>setup.py</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Setuptools shim.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Makefile</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Convenience make targets.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>start.*</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>App launchers (Python/shell/batch).</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>backend_api.py</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Backend ASGI entry point.</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>kill_backend.py</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Utility to free the backend port.</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>.github/**/*</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>GitHub Actions CI workflow.</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>.gitignore</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Git ignore rules.</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>data/raw/cityflowv2/**/*</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Datasets (ground truth)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Copied</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>CityFlowV2 ground-truth / seqinfo for eval.</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>From the external CityFlowV2 / AI City Challenge 2022 dataset (full dataset not included).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(submission): apply LLM/handwritten authorship split to Project Code.xlsx
Mark as "Generated by LLM" per author: wildtrack_calibration, stage0+stage5
format_converter, robust_pool, graph_solver, report_generator, video_annotator,
nl_query, simulation_3d; all docs/*.md; and all non-stage tests. Stage tests
(test_stage0-5, wildtrack_mvdetr, stage2_features) stay Original (handwritten).
reranking.py and query_expansion.py confirmed Original (own implementations of
cited algorithms, not copied). 65 rows, verified 100% file coverage.
</commit_message>
<xml_diff>
--- a/Project Code.xlsx
+++ b/Project Code.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Project" sheetId="1" state="visible" r:id="rId1"/>
@@ -164,32 +164,6 @@
   </cellStyles>
   <dxfs count="7">
     <dxf>
-      <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <b val="1"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <condense val="0"/>
-        <color theme="0"/>
-        <extend val="0"/>
-        <sz val="11"/>
-        <vertAlign val="baseline"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
@@ -226,6 +200,32 @@
         <top/>
         <bottom/>
       </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <b val="1"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <condense val="0"/>
+        <color theme="0"/>
+        <extend val="0"/>
+        <sz val="11"/>
+        <vertAlign val="baseline"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -301,12 +301,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Modules" displayName="Modules" ref="A9:D30" headerRowCount="1" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="5" tableBorderDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Modules" displayName="Modules" ref="A9:D30" headerRowCount="1" totalsRowShown="0" headerRowDxfId="4" headerRowBorderDxfId="3" tableBorderDxfId="2">
   <autoFilter ref="A9:D30"/>
   <tableColumns count="4">
-    <tableColumn id="1" name="Module Name" dataDxfId="3"/>
+    <tableColumn id="1" name="Module Name" dataDxfId="1"/>
     <tableColumn id="2" name="Module Description (Briefly describe what it does and how it works)"/>
-    <tableColumn id="3" name="Module Type" dataDxfId="2"/>
+    <tableColumn id="3" name="Module Type" dataDxfId="0"/>
     <tableColumn id="4" name="Comments (Optional)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -314,12 +314,15 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table3" displayName="Table3" ref="A1:E1001" headerRowCount="1" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A1:E1001"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table3" displayName="Table3" ref="A1:E1000" headerRowCount="1" totalsRowShown="0" headerRowDxfId="6">
+  <autoFilter ref="A1:E1000"/>
+  <sortState ref="A2:E48">
+    <sortCondition ref="C1:C1000"/>
+  </sortState>
   <tableColumns count="5">
     <tableColumn id="1" name="File Path (Relative to the Project Root, Glob patterns are allowed)"/>
     <tableColumn id="5" name="Module Name"/>
-    <tableColumn id="2" name="Source" dataDxfId="0"/>
+    <tableColumn id="2" name="Source" dataDxfId="5"/>
     <tableColumn id="3" name="Purpose"/>
     <tableColumn id="4" name="Comments (Optional)"/>
   </tableColumns>
@@ -627,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29.5703125" customWidth="1" style="12" min="1" max="1"/>
@@ -981,6 +984,11 @@
           <t>Original</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nl_query.py and simulation_3d.py LLM-generated; the Streamlit dashboards are handwritten.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1103,6 +1111,11 @@
           <t>Original</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Stage tests (test_stage0-5, wildtrack_mvdetr, stage2_features) handwritten; all other tests LLM-generated.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1139,7 +1152,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Unoriginal</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>All docs and .md files are LLM-generated; LICENSE is a standard template.</t>
         </is>
       </c>
     </row>
@@ -1165,6 +1183,15 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A8:D8"/>
@@ -1183,12 +1210,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.140625" customWidth="1" style="12" min="1" max="1"/>
     <col width="21" customWidth="1" style="12" min="2" max="2"/>
-    <col width="12.42578125" customWidth="1" style="1" min="3" max="3"/>
+    <col width="16.5703125" customWidth="1" style="1" min="3" max="3"/>
     <col width="50.42578125" bestFit="1" customWidth="1" style="12" min="4" max="4"/>
     <col width="223.85546875" bestFit="1" customWidth="1" style="12" min="5" max="5"/>
   </cols>
@@ -1223,56 +1250,61 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>src/__init__.py</t>
+          <t>frontend/src/hooks/use-toast.ts</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Frontend Dashboard</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Copied</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Top-level src package marker.</t>
+          <t>Toast notification hook.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>COPIED: the shadcn/ui use-toast hook (adapted from react-hot-toast).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>src/core/**/*</t>
+          <t>src/training/losses.py</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>ReID Training</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Copied</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Shared data models, config loading, IO utilities.</t>
+          <t>ReID loss functions.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bespoke; io_utils numpy-JSON encoder, video_utils FourCC decode, and wildtrack_calibration (cv2 projectPoints/Rodrigues + WILDTRACK grid) use standard OpenCV/numpy idioms.</t>
+          <t>COPIED: Triplet/Center/CE-label-smoothing/Circle losses follow the canonical BoT reference implementations (Luo et al. reid-strong-baseline; Center loss Wen et al.).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>src/stage0_ingestion/**/*</t>
+          <t>src/stage0_ingestion/preprocessor.py</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1282,29 +1314,29 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Frame extraction and preprocessing.</t>
+          <t>Frame preprocessing (CLAHE, denoise).</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Bespoke; format_converter follows the MOTChallenge/WILDTRACK annotation schemas.</t>
+          <t>MIXED: LAB-channel CLAHE block follows the OpenCV tutorial recipe; surrounding pipeline bespoke.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>src/stage0_ingestion/preprocessor.py</t>
+          <t>src/stage2_features/transreid_model.py</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Stage 0 - Ingestion</t>
+          <t>Stage 2 - Features</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1314,46 +1346,46 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Frame preprocessing (CLAHE, denoise).</t>
+          <t>TransReID model for inference.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>MIXED: the LAB-channel CLAHE block follows the canonical OpenCV tutorial recipe; surrounding pipeline is bespoke.</t>
+          <t>MIXED: SIE/JPM/BNNeck follow the official TransReID architecture (He et al., ICCV 2021); timm/CLIP integration bespoke.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>src/stage1_tracking/**/*</t>
+          <t>src/stage2_features/clip_senet_model.py</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Stage 1 - Tracking</t>
+          <t>Stage 2 - Features</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>YOLO detection + BoxMOT tracking.</t>
+          <t>CLIP-SENet vehicle ReID model.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Glue/wrappers around Ultralytics YOLO and BoxMOT (BoT-SORT); IoU + linear interpolation are textbook helpers; rest bespoke.</t>
+          <t>MIXED: AFEM/architecture ported from the CLIP-SENet paper; backbones via torch.hub/open_clip; assembly bespoke.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>src/stage2_features/**/*</t>
+          <t>src/stage2_features/foreground_masker.py</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1363,24 +1395,24 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ReID embeddings, HSV, PCA.</t>
+          <t>SAM2 foreground masking.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Bespoke; pca_whitening wraps sklearn PCA, hsv_extractor uses cv2.calcHist, reid_model state-dict remaps are keyed to fast-reid/IBN-Net layouts.</t>
+          <t>MIXED: SAM2 point-prompt inference follows the official SAM2 model-card usage; registry/loader bespoke.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>src/stage2_features/transreid_model.py</t>
+          <t>src/stage2_features/foreground_masking.py</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1395,24 +1427,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>TransReID model for inference.</t>
+          <t>SAM2 automatic-mask masking.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>MIXED: SIE/JPM/BNNeck follow the official TransReID architecture (He et al., ICCV 2021); timm/CLIP integration + weight remapping bespoke.</t>
+          <t>MIXED: SAM2 automatic-mask-generator usage from the SAM2 README; plumbing bespoke.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>src/stage2_features/clip_senet_model.py</t>
+          <t>src/stage4_association/fic.py</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Stage 2 - Features</t>
+          <t>Stage 4 - Association</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1422,24 +1454,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CLIP-SENet vehicle ReID model.</t>
+          <t>Per-camera FIC whitening.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>MIXED: AFEM/architecture ported from the CLIP-SENet paper; backbones via torch.hub/open_clip; assembly bespoke.</t>
+          <t>MIXED: per-camera whitening adapted from the AIC21 1st-place ficfac.py (Liu et al., CVPRW 2021).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>src/stage2_features/foreground_masker.py</t>
+          <t>src/training/model.py</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Stage 2 - Features</t>
+          <t>ReID Training</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1449,24 +1481,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>SAM2 foreground masking.</t>
+          <t>BoT ReID backbone.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>MIXED: SAM2 point-prompt inference follows the official SAM2 model-card usage; registry/loader bespoke (default-off experimental).</t>
+          <t>MIXED: IBN-a from XingangPan/IBN-Net + BNNeck from BoT (canonical); build/loading bespoke.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>src/stage2_features/foreground_masking.py</t>
+          <t>src/training/evaluate_reid.py</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Stage 2 - Features</t>
+          <t>ReID Training</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1476,397 +1508,402 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SAM2 automatic-mask masking.</t>
+          <t>ReID evaluation (CMC/mAP) + re-ranking.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>MIXED: SAM2 automatic-mask-generator usage from the SAM2 README; plumbing bespoke (default-off experimental).</t>
+          <t>MIXED: eval_market1501 (CMC/mAP) and compute_reranking (k-reciprocal, Zhong et al. 2017) follow canonical reference code; orchestration bespoke.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>src/stage3_indexing/**/*</t>
+          <t>backend/services/reid_service.py</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Stage 3 - Indexing</t>
+          <t>Backend API</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FAISS index and SQLite metadata.</t>
+          <t>ReID inference service.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Glue/wrapper around FAISS + SQLite (idiomatic API usage).</t>
+          <t>MIXED: the dense _compute_reranking is the canonical k-reciprocal algorithm (Zhong et al. 2017); rest bespoke.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>src/stage4_association/**/*</t>
+          <t>frontend/src/lib/utils.ts</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Stage 4 - Association</t>
+          <t>Frontend Dashboard</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Cross-camera association graph and solver.</t>
+          <t>Frontend utility helpers.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Bespoke reimplementations; AQE/k-reciprocal/AFLink/camera-bias/zone cite their techniques in headers (verified not line-level ports).</t>
+          <t>MIXED: cn() (shadcn), debounce/throttle/formatBytes/getCameraColor are common tutorial/Stack-Overflow snippets; other helpers bespoke.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>src/stage4_association/fic.py</t>
+          <t>src/core/wildtrack_calibration.py</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Stage 4 - Association</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Generated by LLM</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Per-camera FIC whitening.</t>
+          <t>WILDTRACK camera calibration parsing/projection.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MIXED: per-camera whitening adapted from the AIC21 1st-place ficfac.py (Liu et al., CVPRW 2021); wrappers bespoke.</t>
+          <t>Generated with an LLM.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>src/stage5_evaluation/**/*</t>
+          <t>src/stage0_ingestion/format_converter.py</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Stage 5 - Evaluation</t>
+          <t>Stage 0 - Ingestion</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Generated by LLM</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Metrics and format conversion.</t>
+          <t>MOT/WILDTRACK annotation format conversion.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Glue/wrapper around TrackEval + py-motmetrics.</t>
+          <t>Generated with an LLM.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>src/stage6_visualization/**/*</t>
+          <t>src/stage2_features/robust_pool.py</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Stage 6 - Visualization</t>
+          <t>Stage 2 - Features</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Generated by LLM</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Annotated video, BEV, timeline.</t>
+          <t>Robust tracklet feature pooling (geometric median etc.).</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Bespoke; standard matplotlib/Plotly palettes and cv2 drawing idioms.</t>
+          <t>Generated with an LLM.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>src/stage_wildtrack_mvdetr/**/*</t>
+          <t>src/stage4_association/graph_solver.py</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>WILDTRACK MVDeTr</t>
+          <t>Stage 4 - Association</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Generated by LLM</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Ground-plane person detection + tracking.</t>
+          <t>Graph-based identity clustering solver.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Bespoke glue; constant-velocity Kalman is the textbook DWNA model; WILDTRACK grid constants are dataset facts; consumes external MVDeTr outputs.</t>
+          <t>Generated with an LLM.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>src/training/**/*</t>
+          <t>src/stage5_evaluation/format_converter.py</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ReID Training</t>
+          <t>Stage 5 - Evaluation</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Generated by LLM</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Training loops, datasets, seeding.</t>
+          <t>MOTChallenge format conversion for evaluation.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Bespoke trainer; datasets/seed/train_reid follow the standard BoT recipe + PyTorch reproducibility idioms (independently written). See per-file rows.</t>
+          <t>Generated with an LLM.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>src/training/losses.py</t>
+          <t>src/stage5_evaluation/report_generator.py</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ReID Training</t>
+          <t>Stage 5 - Evaluation</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Copied</t>
+          <t>Generated by LLM</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>ReID loss functions.</t>
+          <t>Evaluation report generation.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>COPIED: Triplet/Center/CE-label-smoothing/Circle losses follow the canonical BoT reference implementations (Luo et al. reid-strong-baseline; Center loss Wen et al.).</t>
+          <t>Generated with an LLM.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>src/training/model.py</t>
+          <t>src/stage6_visualization/video_annotator.py</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ReID Training</t>
+          <t>Stage 6 - Visualization</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Generated by LLM</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>BoT ReID backbone.</t>
+          <t>Annotated-video rendering.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>MIXED: IBN-a from XingangPan/IBN-Net + BNNeck from BoT (canonical); build/loading bespoke; loads IBN-Net weights by URL.</t>
+          <t>Generated with an LLM.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>src/training/evaluate_reid.py</t>
+          <t>src/apps/nl_query.py</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ReID Training</t>
+          <t>Auxiliary Apps</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Generated by LLM</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ReID evaluation (CMC/mAP) + re-ranking.</t>
+          <t>Natural-language query interface.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>MIXED: eval_market1501 (CMC/mAP) and compute_reranking (k-reciprocal, Zhong et al. 2017) follow canonical Market-1501/reid reference code; orchestration bespoke.</t>
+          <t>Generated with an LLM.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>src/serving/**/*</t>
+          <t>src/apps/simulation_3d.py</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Model Serving</t>
+          <t>Auxiliary Apps</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Generated by LLM</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>ReID model loaders and cache.</t>
+          <t>3D simulation viewer.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Loaders/glue around torch/timm/open_clip; CLIP/ImageNet normalization are the standard published constants.</t>
+          <t>Generated with an LLM.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>src/apps/**/*</t>
+          <t>LICENSE</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Auxiliary Apps</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Original from Template</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Streamlit dashboard, NL query, 3D sim.</t>
+          <t>MIT license.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Standard MIT License text.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>backend/**/*</t>
+          <t>Project Code.xlsx</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Backend API</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Original from Template</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>FastAPI service, routers, services, registry.</t>
+          <t>This submission spreadsheet.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Bespoke FastAPI application (framework idioms are normal usage).</t>
+          <t>Course-provided template, filled in by us.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>backend/services/reid_service.py</t>
+          <t>frontend/src/components/ui/**/*</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Backend API</t>
+          <t>Frontend UI Primitives</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Copied</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>ReID inference service.</t>
+          <t>Reusable UI primitives.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>MIXED: the dense _compute_reranking is the canonical k-reciprocal algorithm (Zhong et al. 2017); image handling/AQE/fusion/scoring bespoke.</t>
+          <t>Generated by the shadcn/ui CLI (https://ui.shadcn.com/) - not written by us.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>frontend/src/components/ui/**/*</t>
+          <t>data/raw/cityflowv2/**/*</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Frontend UI Primitives</t>
+          <t>Datasets (ground truth)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1876,132 +1913,132 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Reusable UI primitives.</t>
+          <t>CityFlowV2 ground-truth / seqinfo for eval.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Generated by the shadcn/ui CLI (https://ui.shadcn.com/), built on Radix UI - not written by us.</t>
+          <t>From the external CityFlowV2 / AI City Challenge 2022 dataset.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>frontend/src/hooks/use-toast.ts</t>
+          <t>scripts/eval/**/*</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Frontend Dashboard</t>
+          <t>Scripts and Tooling</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Copied</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Toast notification hook.</t>
+          <t>VeRi-776 ReID evaluation modules.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>COPIED: the shadcn/ui use-toast hook (adapted from react-hot-toast).</t>
+          <t>MIXED: compute_reranking_torch (k-reciprocal) + eval_market1501 (CMC/mAP) are canonical reference code; CLI/plumbing bespoke.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>frontend/src/lib/utils.ts</t>
+          <t>docs/**/*</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Frontend Dashboard</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Generated by LLM</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Frontend utility helpers.</t>
+          <t>Architecture, dataset, model-card docs.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>MIXED: cn() (shadcn), debounce/throttle/formatBytes/getCameraColor are common tutorial/Stack-Overflow snippets; other helpers bespoke.</t>
+          <t>Generated with an LLM.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>frontend/**/*</t>
+          <t>models/**/*</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Frontend Dashboard</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Generated by LLM</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Next.js ATHAR dashboard app, hooks, store, API client.</t>
+          <t>Model-weights README / placement instructions.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Excludes components/ui/** and the two files above. Root config (next.config, tsconfig, tailwind, components.json, package.json) scaffolded by create-next-app + shadcn init and customized by us; next-env.d.ts/package-lock.json auto-generated.</t>
+          <t>Generated with an LLM. Checkpoints not included (gitignored).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>configs/**/*</t>
+          <t>*.md</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Configuration</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Generated by LLM</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>OmegaConf pipeline/dataset/model configs.</t>
+          <t>README, SETUP, LAUNCH and other markdown docs.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Hand-tuned.</t>
+          <t>Generated with an LLM.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>scripts/**/*</t>
+          <t>tests/test_stage0/**/*</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Tests</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2011,46 +2048,46 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CLI entry points, asset download/verify, helpers.</t>
+          <t>Stage 0 tests.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Bespoke; see scripts/eval row.</t>
+          <t>Handwritten.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>scripts/eval/**/*</t>
+          <t>tests/test_stage1/**/*</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Tests</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>VeRi-776 ReID evaluation modules.</t>
+          <t>Stage 1 tests.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>MIXED: compute_reranking_torch (k-reciprocal, Zhong et al. 2017) and eval_market1501 (CMC/mAP) are canonical ReID reference code; model defs + CLI/JSON plumbing bespoke.</t>
+          <t>Handwritten.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>tests/**/*</t>
+          <t>tests/test_stage2/**/*</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2065,46 +2102,51 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Pytest suite across stages, backend, scripts.</t>
+          <t>Stage 2 tests.</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Handwritten.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>notebooks/**/*</t>
+          <t>tests/test_stage3/**/*</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Kaggle Notebooks</t>
+          <t>Tests</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Original from Template</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>GPU training/pipeline/verification runners.</t>
+          <t>Stage 3 tests.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Generated from templates by the project's notebook-builder tooling; wrap src/ pipeline code.</t>
+          <t>Handwritten.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>docs/**/*</t>
+          <t>tests/test_stage4/**/*</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Tests</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2114,19 +2156,24 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Architecture, dataset, model-card docs.</t>
+          <t>Stage 4 tests.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Handwritten.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>*.md</t>
+          <t>tests/test_stage5/**/*</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Tests</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2136,46 +2183,51 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Top-level README, SETUP, LAUNCH guides.</t>
+          <t>Stage 5 tests.</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Handwritten.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>LICENSE</t>
+          <t>tests/test_stage_wildtrack_mvdetr/**/*</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Tests</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Original from Template</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>MIT license.</t>
+          <t>WILDTRACK MVDeTr stage tests.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Standard MIT License text.</t>
+          <t>Handwritten.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>models/**/*</t>
+          <t>tests/stage2_features/**/*</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Tests</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2185,78 +2237,78 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Model-weights README / placement instructions.</t>
+          <t>Stage 2 feature tests.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Checkpoints themselves are not included (gitignored); see README.</t>
+          <t>Handwritten.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Project Code.xlsx</t>
+          <t>tests/**/*</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Tests</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Original from Template</t>
+          <t>Generated by LLM</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>This submission spreadsheet.</t>
+          <t>Backend/core/integration/scripts/setup tests + fixtures.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Course-provided template, filled in by us.</t>
+          <t>Generated with an LLM.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>*requirements.txt</t>
+          <t>notebooks/**/*</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Kaggle Notebooks</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Original from Template</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Python dependency manifests.</t>
+          <t>GPU training/pipeline/verification runners.</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>List external pip dependencies (not vendored).</t>
+          <t>Generated from templates by the project's notebook-builder tooling.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>pyproject.toml</t>
+          <t>src/__init__.py</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2266,19 +2318,20 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Build config and project metadata.</t>
-        </is>
-      </c>
+          <t>Top-level src package marker.</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>setup.py</t>
+          <t>src/core/**/*</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2288,19 +2341,24 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Setuptools shim.</t>
+          <t>Shared data models, config, IO utilities.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Bespoke (standard numpy/OpenCV idioms in places).</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Makefile</t>
+          <t>src/stage0_ingestion/**/*</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Stage 0 - Ingestion</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2310,19 +2368,24 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Convenience make targets.</t>
+          <t>Frame extraction and preprocessing.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Bespoke.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>start.*</t>
+          <t>src/stage1_tracking/**/*</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Stage 1 - Tracking</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2332,19 +2395,24 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>App launchers (Python/shell/batch).</t>
+          <t>YOLO detection + BoxMOT tracking.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Glue/wrappers around Ultralytics YOLO and BoxMOT (BoT-SORT).</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>backend_api.py</t>
+          <t>src/stage2_features/**/*</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Stage 2 - Features</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2354,19 +2422,24 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Backend ASGI entry point.</t>
+          <t>ReID embeddings, HSV, PCA.</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Bespoke; pca wraps sklearn, hsv uses cv2.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>kill_backend.py</t>
+          <t>src/stage3_indexing/**/*</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Stage 3 - Indexing</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2376,19 +2449,24 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Utility to free the backend port.</t>
+          <t>FAISS index + SQLite metadata.</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Glue/wrapper around FAISS + SQLite.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>.github/**/*</t>
+          <t>src/stage4_association/**/*</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Stage 4 - Association</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2398,19 +2476,24 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>GitHub Actions CI workflow.</t>
+          <t>Cross-camera association graph and solver.</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Bespoke; reranking/AQE/camera-bias are own implementations of cited algorithms (not copied).</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>.gitignore</t>
+          <t>src/stage5_evaluation/**/*</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Scripts and Tooling</t>
+          <t>Stage 5 - Evaluation</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2420,40 +2503,468 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Git ignore rules.</t>
+          <t>Metrics and evaluation.</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Glue/wrapper around TrackEval + py-motmetrics.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>data/raw/cityflowv2/**/*</t>
+          <t>src/stage6_visualization/**/*</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Datasets (ground truth)</t>
+          <t>Stage 6 - Visualization</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Copied</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>CityFlowV2 ground-truth / seqinfo for eval.</t>
+          <t>Annotated video, BEV, timeline.</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>From the external CityFlowV2 / AI City Challenge 2022 dataset (full dataset not included).</t>
-        </is>
-      </c>
+          <t>Bespoke; standard cv2/matplotlib idioms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>src/stage_wildtrack_mvdetr/**/*</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>WILDTRACK MVDeTr</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Ground-plane person detection + tracking.</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Bespoke glue; textbook Kalman; consumes external MVDeTr outputs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>src/training/**/*</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ReID Training</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Training loops, datasets, seeding.</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Bespoke trainer (standard BoT recipe).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>src/serving/**/*</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Model Serving</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ReID model loaders and cache.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Loaders/glue around torch/timm/open_clip.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>src/apps/**/*</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Auxiliary Apps</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Streamlit dashboards.</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Bespoke (nl_query/simulation_3d are LLM - see rows above).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>backend/**/*</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Backend API</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>FastAPI service, routers, services, registry.</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Bespoke FastAPI application.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>frontend/**/*</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Frontend Dashboard</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Next.js ATHAR dashboard app.</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Excludes components/ui (shadcn), use-toast/utils (see rows), and *.md. Root config scaffolded by create-next-app + shadcn init.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>configs/**/*</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Configuration</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>OmegaConf pipeline/dataset/model configs.</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Hand-tuned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>scripts/**/*</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>CLI entry points, asset download/verify, helpers.</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Bespoke (scripts/eval is Mixed - see row above).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>*requirements.txt</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Python dependency manifests.</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>pyproject.toml</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Build config and project metadata.</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>setup.py</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Setuptools shim.</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Makefile</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Convenience make targets.</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>start.*</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>App launchers (Python/shell/batch).</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>backend_api.py</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Backend ASGI entry point.</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>kill_backend.py</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Utility to free the backend port.</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>.github/**/*</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>GitHub Actions CI workflow.</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>.gitignore</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Scripts and Tooling</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Git ignore rules.</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>INDIRECT("Modules[Module Name]")</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(submission): update Project sheet + add Key sheet to Project Code.xlsx
- Add a "Key" sheet defining each Source label as used (Original/Handwritten,
  Generated by LLM, Mixed, Copied, Original from Template), incl. the
  non-standard "Mixed".
- Project sheet: add authorship-by-line-count summary to Comments, fix Kaggle
  Notebooks module type to Unoriginal (template/tool-generated), note the new
  handwritten geospatial component under Stage 4.
</commit_message>
<xml_diff>
--- a/Project Code.xlsx
+++ b/Project Code.xlsx
@@ -9,6 +9,7 @@
     <sheet name="Project" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Files" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Option Tables" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Key" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +42,13 @@
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -118,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -158,6 +166,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -703,7 +719,8 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Pre-trained models (the COCO-pretrained YOLO26m detector and the DINOv2 / CLIP backbones) and the project's trained ReID checkpoints all run locally on the same machine. Model checkpoints are large and are not included in the submission; they are downloaded with scripts/download_weights.py (from a public Kaggle dataset, SHA-256 pinned in configs/weights_manifest.yaml) or regenerated with the training notebooks under notebooks/kaggle/. No online or hosted ML APIs are called at runtime.</t>
+          <t>Pre-trained models (the COCO-pretrained YOLO26m detector and the DINOv2 / CLIP backbones) and the project's trained ReID checkpoints all run locally on the same machine. Model checkpoints are large and are not included in the submission; they are downloaded with scripts/download_weights.py (from a public Kaggle dataset, SHA-256 pinned in configs/weights_manifest.yaml) or regenerated with the training notebooks under notebooks/kaggle/. No online or hosted ML APIs are called at runtime.
+Authorship by line count (see Files sheet Source column + the Key sheet for definitions): Original/handwritten 78.2%, Generated by LLM 11.1%, Mixed 7.9%, Copied 2.4%, Original from Template 0.5%.</t>
         </is>
       </c>
     </row>
@@ -859,7 +876,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Bespoke reimplementations (reranking/aflink verified not ports); fic.py adapted from AIC21 ficfac.py.</t>
+          <t>Bespoke reimplementations (reranking/aflink verified not ports); fic.py adapted from AIC21 ficfac.py; geospatial.py is a handwritten reachability component.</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1147,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Unoriginal</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2321,7 +2338,6 @@
           <t>Top-level src package marker.</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2776,7 +2792,6 @@
           <t>Python dependency manifests.</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2799,7 +2814,6 @@
           <t>Build config and project metadata.</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2822,7 +2836,6 @@
           <t>Setuptools shim.</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2845,7 +2858,6 @@
           <t>Convenience make targets.</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2868,7 +2880,6 @@
           <t>App launchers (Python/shell/batch).</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2891,7 +2902,6 @@
           <t>Backend ASGI entry point.</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2914,7 +2924,6 @@
           <t>Utility to free the backend port.</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2937,7 +2946,6 @@
           <t>GitHub Actions CI workflow.</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2960,7 +2968,6 @@
           <t>Git ignore rules.</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -3165,4 +3172,101 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" style="12" min="1" max="1"/>
+    <col width="95" customWidth="1" style="12" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Key - Source labels used in the Files sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>Source label</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Original (Handwritten)</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Written by the team by hand. No code taken from any repository or website, and not AI-generated. These are the files that get checked for plagiarism and count as the team's authored work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Generated by LLM</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>Written or generated with an AI coding assistant (e.g. Claude / Copilot). Disclosed honestly; per the rubric these are skipped by the plagiarism check and are not claimed as hand-authored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>The file contains BOTH team-written code AND code adapted/derived from an external source - a public repository, a published paper's reference implementation, or a tutorial. The external source is named in the file's Comments. (Note: 'Mixed' is not one of the five standard dropdown options; it is used here to flag part-bespoke / part-external files. Treat it as Copied for plagiarism-check purposes.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Copied</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>The file content is copied from an external source and is not the team's work (e.g. shadcn/ui CLI output, external-dataset ground-truth files). The source is named in the file's Comments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Original from Template</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Started from a template or scaffold and filled in / extended by the team - e.g. the create-next-app + shadcn project scaffold, the standard MIT LICENSE text, the Kaggle notebook templates, and this course-provided spreadsheet.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>